<commit_message>
V0.3.8 player review and match-day participation refinement
Approved physical iPad acceptance checkpoint. Validation: 257 unit tests, 124 browser/E2E tests and production build passed. No release tag.
</commit_message>
<xml_diff>
--- a/tests/fixtures/squad-template/Club-21.xlsx
+++ b/tests/fixtures/squad-template/Club-21.xlsx
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:A41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -508,11 +508,6 @@
           <t>Player Name *</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Default No.</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -663,79 +658,60 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n"/>
-      <c r="B23" s="1" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n"/>
-      <c r="B24" s="1" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n"/>
-      <c r="B25" s="1" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n"/>
-      <c r="B26" s="1" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n"/>
-      <c r="B27" s="1" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n"/>
-      <c r="B28" s="1" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n"/>
-      <c r="B29" s="1" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n"/>
-      <c r="B30" s="1" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n"/>
-      <c r="B31" s="1" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n"/>
-      <c r="B32" s="1" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n"/>
-      <c r="B33" s="1" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n"/>
-      <c r="B34" s="1" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n"/>
-      <c r="B35" s="1" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n"/>
-      <c r="B36" s="1" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n"/>
-      <c r="B37" s="1" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n"/>
-      <c r="B38" s="1" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n"/>
-      <c r="B39" s="1" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n"/>
-      <c r="B40" s="1" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n"/>
-      <c r="B41" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>